<commit_message>
Changes made to table
Made a typo on the Lotterman 1000m meta-analysis upper odds-ratio
</commit_message>
<xml_diff>
--- a/Data/Oddsratios.xlsx
+++ b/Data/Oddsratios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marcj\Documents\MSJ\Projects\2025\Bennie Aarts\Subrapport\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15EE7111-8248-402F-BB32-629347718814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E01DCD7D-265E-4BAF-8D04-B568C4C9EF68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3030" yWindow="3030" windowWidth="38700" windowHeight="15105" xr2:uid="{47145107-9674-4BE4-8D57-8645EDA7E158}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{47145107-9674-4BE4-8D57-8645EDA7E158}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -696,27 +696,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB0A062-2371-42C7-9960-6D188BFBC7A3}">
   <dimension ref="A1:S90"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="13" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="1"/>
-    <col min="4" max="5" width="16.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.41796875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.15625" style="1"/>
+    <col min="4" max="5" width="16.68359375" style="1" customWidth="1"/>
     <col min="6" max="6" width="21" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="38.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" style="1" customWidth="1"/>
-    <col min="11" max="12" width="14.140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="13.5703125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="22.85546875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="17.5703125" style="1" customWidth="1"/>
-    <col min="16" max="17" width="9.140625" style="1"/>
-    <col min="18" max="18" width="23.28515625" style="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.140625" style="1"/>
+    <col min="7" max="7" width="12.26171875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="20.68359375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="38.41796875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="11.68359375" style="1" customWidth="1"/>
+    <col min="11" max="12" width="14.15625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13.578125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="22.83984375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="17.578125" style="1" customWidth="1"/>
+    <col min="16" max="17" width="9.15625" style="1"/>
+    <col min="18" max="18" width="23.26171875" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.15625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -775,7 +775,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -831,7 +831,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -884,7 +884,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -937,7 +937,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -990,7 +990,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -1043,7 +1043,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -1096,7 +1096,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1146,7 +1146,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -1196,7 +1196,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
@@ -1296,7 +1296,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
@@ -1346,7 +1346,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="R13" s="2"/>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="R14" s="2"/>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
@@ -1447,7 +1447,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
@@ -1497,7 +1497,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="1" t="s">
         <v>4</v>
       </c>
@@ -1547,7 +1547,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="1" t="s">
         <v>11</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="1" t="s">
         <v>11</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="1" t="s">
         <v>11</v>
       </c>
@@ -1706,7 +1706,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="1" t="s">
         <v>11</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="1" t="s">
         <v>11</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="1" t="s">
         <v>11</v>
       </c>
@@ -1865,7 +1865,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="1" t="s">
         <v>11</v>
       </c>
@@ -1918,7 +1918,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="1" t="s">
         <v>11</v>
       </c>
@@ -1971,7 +1971,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="1" t="s">
         <v>11</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="1" t="s">
         <v>11</v>
       </c>
@@ -2077,7 +2077,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="1" t="s">
         <v>11</v>
       </c>
@@ -2130,7 +2130,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="1" t="s">
         <v>11</v>
       </c>
@@ -2183,7 +2183,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="1" t="s">
         <v>12</v>
       </c>
@@ -2233,7 +2233,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="1" t="s">
         <v>12</v>
       </c>
@@ -2283,7 +2283,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="1" t="s">
         <v>12</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="1" t="s">
         <v>13</v>
       </c>
@@ -2383,7 +2383,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="1" t="s">
         <v>13</v>
       </c>
@@ -2433,7 +2433,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="1" t="s">
         <v>13</v>
       </c>
@@ -2483,7 +2483,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="1" t="s">
         <v>13</v>
       </c>
@@ -2533,7 +2533,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="1" t="s">
         <v>13</v>
       </c>
@@ -2586,7 +2586,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="1" t="s">
         <v>13</v>
       </c>
@@ -2639,7 +2639,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="1" t="s">
         <v>13</v>
       </c>
@@ -2692,7 +2692,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="1" t="s">
         <v>13</v>
       </c>
@@ -2745,7 +2745,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" s="1" t="s">
         <v>13</v>
       </c>
@@ -2789,7 +2789,7 @@
         <v>1</v>
       </c>
       <c r="Q41" s="1">
-        <v>1.1399999999999999</v>
+        <v>1.41</v>
       </c>
       <c r="R41" s="2">
         <v>0.95</v>
@@ -2798,7 +2798,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="1" t="s">
         <v>13</v>
       </c>
@@ -2851,7 +2851,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="1" t="s">
         <v>14</v>
       </c>
@@ -2904,7 +2904,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="1" t="s">
         <v>14</v>
       </c>
@@ -2957,7 +2957,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="1" t="s">
         <v>14</v>
       </c>
@@ -3010,7 +3010,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="1" t="s">
         <v>14</v>
       </c>
@@ -3063,7 +3063,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="1" t="s">
         <v>14</v>
       </c>
@@ -3116,7 +3116,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="1" t="s">
         <v>14</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="1" t="s">
         <v>14</v>
       </c>
@@ -3222,7 +3222,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="1" t="s">
         <v>14</v>
       </c>
@@ -3275,7 +3275,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="1" t="s">
         <v>14</v>
       </c>
@@ -3328,7 +3328,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="1" t="s">
         <v>14</v>
       </c>
@@ -3381,7 +3381,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="1" t="s">
         <v>14</v>
       </c>
@@ -3434,7 +3434,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="1" t="s">
         <v>14</v>
       </c>
@@ -3487,7 +3487,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="1" t="s">
         <v>14</v>
       </c>
@@ -3543,7 +3543,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="1" t="s">
         <v>14</v>
       </c>
@@ -3599,7 +3599,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="1" t="s">
         <v>14</v>
       </c>
@@ -3655,7 +3655,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="1" t="s">
         <v>14</v>
       </c>
@@ -3711,7 +3711,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="1" t="s">
         <v>14</v>
       </c>
@@ -3767,7 +3767,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="1" t="s">
         <v>14</v>
       </c>
@@ -3823,7 +3823,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="1" t="s">
         <v>14</v>
       </c>
@@ -3879,7 +3879,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="1" t="s">
         <v>14</v>
       </c>
@@ -3935,7 +3935,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="1" t="s">
         <v>14</v>
       </c>
@@ -3991,7 +3991,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="1" t="s">
         <v>14</v>
       </c>
@@ -4047,7 +4047,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="1" t="s">
         <v>14</v>
       </c>
@@ -4103,7 +4103,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="1" t="s">
         <v>14</v>
       </c>
@@ -4159,7 +4159,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="1" t="s">
         <v>14</v>
       </c>
@@ -4215,7 +4215,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="1" t="s">
         <v>14</v>
       </c>
@@ -4271,7 +4271,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="1" t="s">
         <v>14</v>
       </c>
@@ -4327,7 +4327,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="1" t="s">
         <v>14</v>
       </c>
@@ -4383,7 +4383,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="1" t="s">
         <v>14</v>
       </c>
@@ -4439,7 +4439,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="1" t="s">
         <v>14</v>
       </c>
@@ -4495,7 +4495,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="1" t="s">
         <v>14</v>
       </c>
@@ -4551,7 +4551,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" s="1" t="s">
         <v>14</v>
       </c>
@@ -4607,7 +4607,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" s="1" t="s">
         <v>14</v>
       </c>
@@ -4663,7 +4663,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A76" s="1" t="s">
         <v>14</v>
       </c>
@@ -4719,7 +4719,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A77" s="1" t="s">
         <v>14</v>
       </c>
@@ -4775,7 +4775,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A78" s="1" t="s">
         <v>14</v>
       </c>
@@ -4831,7 +4831,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A79" s="1" t="s">
         <v>14</v>
       </c>
@@ -4887,7 +4887,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A80" s="1" t="s">
         <v>14</v>
       </c>
@@ -4943,7 +4943,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A81" s="1" t="s">
         <v>14</v>
       </c>
@@ -4999,7 +4999,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A82" s="1" t="s">
         <v>14</v>
       </c>
@@ -5055,7 +5055,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A83" s="1" t="s">
         <v>14</v>
       </c>
@@ -5111,7 +5111,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A84" s="1" t="s">
         <v>14</v>
       </c>
@@ -5167,7 +5167,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A85" s="1" t="s">
         <v>14</v>
       </c>
@@ -5223,7 +5223,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A86" s="1" t="s">
         <v>14</v>
       </c>
@@ -5279,7 +5279,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A87" s="1" t="s">
         <v>14</v>
       </c>
@@ -5335,7 +5335,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A88" s="1" t="s">
         <v>14</v>
       </c>
@@ -5391,7 +5391,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A89" s="1" t="s">
         <v>14</v>
       </c>
@@ -5447,7 +5447,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A90" s="1" t="s">
         <v>14</v>
       </c>

</xml_diff>